<commit_message>
bug fix and data update for 2019 pipeline capacities
Limit imports to Italy from northern Africa due to north-south bottlenecks in Italy (assumption based).
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/02_paper_ESR/inputs_ESR_2026_run_2019.xlsx
+++ b/01_data/01_input_data/02_processed/02_paper_ESR/inputs_ESR_2026_run_2019.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\02_paper_ESR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{428A52D8-9A1D-456C-9955-9D979D39E813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54CD6CB0-0F2A-489B-9F29-F82202482725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-12975" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -6107,10 +6107,10 @@
         <v>17</v>
       </c>
       <c r="D53">
-        <v>182135</v>
+        <v>60000</v>
       </c>
       <c r="E53">
-        <v>182135</v>
+        <v>60000</v>
       </c>
       <c r="F53">
         <v>3131.085096797216</v>
@@ -6832,10 +6832,10 @@
         <v>17</v>
       </c>
       <c r="D78">
-        <v>421210</v>
+        <v>120000</v>
       </c>
       <c r="E78">
-        <v>421210</v>
+        <v>120000</v>
       </c>
       <c r="F78">
         <v>1736.696056306987</v>

</xml_diff>